<commit_message>
add assertion on login button click
</commit_message>
<xml_diff>
--- a/tests/urls/LogoCheck.xlsx
+++ b/tests/urls/LogoCheck.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joliva\Desktop\PLAYWRIGHT FILES\playwright partner pages\tests\urls\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EABE6A7-0DF4-4CC6-806C-31218280E79E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64F381C7-2B79-4E54-AE6F-8C8C3BF3C6B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="990" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="181">
   <si>
     <t>URL</t>
   </si>
@@ -579,6 +579,12 @@
   </si>
   <si>
     <t>https://ltcrplus.com/</t>
+  </si>
+  <si>
+    <t>https://purdue.ltcrplus.com/?q=123</t>
+  </si>
+  <si>
+    <t>https://usu.ltcrplus.com/</t>
   </si>
 </sst>
 </file>
@@ -1008,6 +1014,22 @@
         <v>27</v>
       </c>
     </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>180</v>
+      </c>
+    </row>
     <row r="45" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B45" s="9"/>
     </row>
@@ -1408,6 +1430,8 @@
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" xr:uid="{770C30FE-8F51-4D26-AA01-1B863C77984B}"/>
     <hyperlink ref="B3" r:id="rId2" xr:uid="{FB2EC7F1-F467-48D7-92B5-0372A20164F4}"/>
+    <hyperlink ref="B4" r:id="rId3" xr:uid="{C4CD68BB-395B-4B14-9962-E37690CD643C}"/>
+    <hyperlink ref="B5" r:id="rId4" xr:uid="{203BE2A5-A4C8-412C-A08B-8DEF29F42440}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Final push by JOLIVA, transferring repo to AJCASTRILLO
</commit_message>
<xml_diff>
--- a/tests/urls/LogoCheck.xlsx
+++ b/tests/urls/LogoCheck.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joliva\Desktop\PLAYWRIGHT FILES\playwright partner pages\tests\urls\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{002CDBF6-A6C6-4D25-BF2B-BF85698400FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1EF4825-54ED-4C0E-AF7E-7233EF443A1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="36150" yWindow="2895" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="178">
   <si>
     <t>URL</t>
   </si>
@@ -576,18 +576,6 @@
   </si>
   <si>
     <t>https://bcf.ltcrplus.com/</t>
-  </si>
-  <si>
-    <t>https://lsus.ltcrplus.com/</t>
-  </si>
-  <si>
-    <t>https://wscaa.ltcrplus.com/</t>
-  </si>
-  <si>
-    <t>https://umem.ltcrplus.com/</t>
-  </si>
-  <si>
-    <t>https://elizc.ltcrplus.com/</t>
   </si>
 </sst>
 </file>
@@ -984,7 +972,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B176"/>
+  <dimension ref="A1:B103"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
@@ -1003,8 +991,8 @@
       <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="7" t="s">
-        <v>178</v>
+      <c r="B2" s="6" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -1012,32 +1000,17 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>179</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>180</v>
-      </c>
+      <c r="B4" s="6"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>181</v>
-      </c>
+      <c r="B5" s="6"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>2</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>24</v>
-      </c>
+      <c r="B6" s="6"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B7" s="6"/>
@@ -1187,7 +1160,7 @@
       <c r="B55" s="6"/>
     </row>
     <row r="56" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B56" s="6"/>
+      <c r="B56" s="9"/>
     </row>
     <row r="57" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B57" s="6"/>
@@ -1220,7 +1193,7 @@
       <c r="B66" s="6"/>
     </row>
     <row r="67" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B67" s="6"/>
+      <c r="B67" s="9"/>
     </row>
     <row r="68" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B68" s="6"/>
@@ -1330,232 +1303,10 @@
     <row r="103" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B103" s="6"/>
     </row>
-    <row r="104" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B104" s="9"/>
-    </row>
-    <row r="105" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B105" s="6"/>
-    </row>
-    <row r="106" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B106" s="6"/>
-    </row>
-    <row r="107" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B107" s="6"/>
-    </row>
-    <row r="108" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B108" s="6"/>
-    </row>
-    <row r="109" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B109" s="6"/>
-    </row>
-    <row r="110" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B110" s="6"/>
-    </row>
-    <row r="111" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B111" s="6"/>
-    </row>
-    <row r="112" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B112" s="6"/>
-    </row>
-    <row r="113" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B113" s="6"/>
-    </row>
-    <row r="114" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B114" s="6"/>
-    </row>
-    <row r="115" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B115" s="6"/>
-    </row>
-    <row r="116" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B116" s="6"/>
-    </row>
-    <row r="117" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B117" s="6"/>
-    </row>
-    <row r="118" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B118" s="6"/>
-    </row>
-    <row r="119" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B119" s="6"/>
-    </row>
-    <row r="120" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B120" s="9"/>
-    </row>
-    <row r="121" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B121" s="9"/>
-    </row>
-    <row r="122" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B122" s="6"/>
-    </row>
-    <row r="123" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B123" s="6"/>
-    </row>
-    <row r="124" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B124" s="6"/>
-    </row>
-    <row r="125" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B125" s="6"/>
-    </row>
-    <row r="126" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B126" s="6"/>
-    </row>
-    <row r="127" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B127" s="6"/>
-    </row>
-    <row r="128" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B128" s="6"/>
-    </row>
-    <row r="129" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B129" s="9"/>
-    </row>
-    <row r="130" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B130" s="6"/>
-    </row>
-    <row r="131" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B131" s="6"/>
-    </row>
-    <row r="132" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B132" s="6"/>
-    </row>
-    <row r="133" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B133" s="6"/>
-    </row>
-    <row r="134" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B134" s="6"/>
-    </row>
-    <row r="135" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B135" s="6"/>
-    </row>
-    <row r="136" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B136" s="6"/>
-    </row>
-    <row r="137" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B137" s="6"/>
-    </row>
-    <row r="138" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B138" s="6"/>
-    </row>
-    <row r="139" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B139" s="6"/>
-    </row>
-    <row r="140" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B140" s="9"/>
-    </row>
-    <row r="141" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B141" s="6"/>
-    </row>
-    <row r="142" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B142" s="6"/>
-    </row>
-    <row r="143" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B143" s="6"/>
-    </row>
-    <row r="144" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B144" s="6"/>
-    </row>
-    <row r="145" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B145" s="6"/>
-    </row>
-    <row r="146" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B146" s="6"/>
-    </row>
-    <row r="147" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B147" s="6"/>
-    </row>
-    <row r="148" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B148" s="6"/>
-    </row>
-    <row r="149" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B149" s="6"/>
-    </row>
-    <row r="150" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B150" s="6"/>
-    </row>
-    <row r="151" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B151" s="6"/>
-    </row>
-    <row r="152" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B152" s="6"/>
-    </row>
-    <row r="153" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B153" s="6"/>
-    </row>
-    <row r="154" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B154" s="6"/>
-    </row>
-    <row r="155" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B155" s="6"/>
-    </row>
-    <row r="156" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B156" s="6"/>
-    </row>
-    <row r="157" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B157" s="6"/>
-    </row>
-    <row r="158" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B158" s="6"/>
-    </row>
-    <row r="159" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B159" s="6"/>
-    </row>
-    <row r="160" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B160" s="6"/>
-    </row>
-    <row r="161" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B161" s="6"/>
-    </row>
-    <row r="162" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B162" s="6"/>
-    </row>
-    <row r="163" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B163" s="6"/>
-    </row>
-    <row r="164" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B164" s="6"/>
-    </row>
-    <row r="165" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B165" s="6"/>
-    </row>
-    <row r="166" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B166" s="6"/>
-    </row>
-    <row r="167" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B167" s="6"/>
-    </row>
-    <row r="168" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B168" s="6"/>
-    </row>
-    <row r="169" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B169" s="6"/>
-    </row>
-    <row r="170" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B170" s="6"/>
-    </row>
-    <row r="171" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B171" s="6"/>
-    </row>
-    <row r="172" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B172" s="6"/>
-    </row>
-    <row r="173" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B173" s="6"/>
-    </row>
-    <row r="174" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B174" s="6"/>
-    </row>
-    <row r="175" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B175" s="6"/>
-    </row>
-    <row r="176" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B176" s="6"/>
-    </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" xr:uid="{BB1E2BE2-37D0-44B2-90C6-E91E439F7ADC}"/>
-    <hyperlink ref="B3" r:id="rId2" xr:uid="{162B3266-180F-407F-9314-446E888AD44A}"/>
-    <hyperlink ref="B4" r:id="rId3" xr:uid="{02FB3888-C806-452C-AC41-B0B4F7D06A0D}"/>
-    <hyperlink ref="B5" r:id="rId4" xr:uid="{6159EA1B-7647-4E59-BFB9-9AE93D27A681}"/>
-    <hyperlink ref="B6" r:id="rId5" xr:uid="{753CACB6-342D-4D4C-A7A3-D1A07D7EFC13}"/>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{9C057366-A70A-44E0-A2CD-75F9893BE95D}"/>
+    <hyperlink ref="B3" r:id="rId2" xr:uid="{F21EF682-B1F4-4DA4-91A1-30447EB4AF79}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>